<commit_message>
Propagate TCM=UNKNOWN bureau correction to Oakland/Equifax/TCM deliverables
https://claude.ai/code/session_014WdfNSevF6i6PT6GydKC2F
</commit_message>
<xml_diff>
--- a/research/alameda/deliverables/Oakland_Business_HardInquiry_v1.xlsx
+++ b/research/alameda/deliverables/Oakland_Business_HardInquiry_v1.xlsx
@@ -501,9 +501,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -657,9 +655,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Flag Metropolitan Bank rail conflict (Elan storefront vs TCM mycommunitycc) in Oakland sheet
https://claude.ai/code/session_014WdfNSevF6i6PT6GydKC2F
</commit_message>
<xml_diff>
--- a/research/alameda/deliverables/Oakland_Business_HardInquiry_v1.xlsx
+++ b/research/alameda/deliverables/Oakland_Business_HardInquiry_v1.xlsx
@@ -501,7 +501,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -655,7 +654,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -1608,12 +1606,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Elan</t>
+          <t>RAIL CONFLICT: Elan (mbonlineportal) vs TCM (mycommunitycc/FROlvrV1uR72) — unresolved</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>follows-rail</t>
+          <t>UNKNOWN — if Elan≈TU-usual; if TCM, bureau undocumented. Confirm at application</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">

</xml_diff>